<commit_message>
auto: snapshot 2026-09-14 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -58,6 +58,7 @@
     <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40089,6 +40090,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-14 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>44711</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2148</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6735</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+2050</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>14499</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>3655</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>34226</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2544</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>896</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+316</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1331</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6457</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>12221</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+2496</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>20477</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+2145</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>9695</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+1317</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3414</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>9721</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+530</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2975</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+1012</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>25577</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+2600</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>7354</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+2757</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>12757</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6586</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+2170</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>23392</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2175</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6642</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+2030</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>15100</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>990</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8427</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1570</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>10294</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>17527</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+2164</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SETYA:)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>15467</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+1210</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>10090</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>30530</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3622</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2377</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>15494</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+520</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>13642</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8483</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+402</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>11113</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+310</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>1029</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>650</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>11377</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1602</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-14 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -40120,11 +40120,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-14 13:00:09</t>
+          <t>Timestamp: 2026-09-14 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>44711</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
@@ -40451,11 +40451,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>7354</v>
+        <v>7405</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+2757</t>
+          <t>+2808</t>
         </is>
       </c>
     </row>
@@ -40631,11 +40631,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>17527</v>
+        <v>17577</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+2164</t>
+          <t>+2214</t>
         </is>
       </c>
     </row>
@@ -40706,11 +40706,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>30530</v>
+        <v>30580</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3622</t>
+          <t>+3672</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -59,6 +59,7 @@
     <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40918,6 +40919,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-15 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>19519</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2148</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6735</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>14799</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>3655</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>36076</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1850</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1046</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1581</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6457</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>12721</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>21691</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>10600</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+905</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3414</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>9721</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>3075</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>27477</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1900</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9402</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6586</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>23392</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>6642</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>15400</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>990</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>8457</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+30</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>10914</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> cassanova98</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>791</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>18768</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1191</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SETYA:)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>16422</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+955</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>10110</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>32726</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+2146</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2618</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+241</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>15794</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>13642</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>9503</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>11413</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>1179</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>12615</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1238</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 05:30:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -40949,11 +40949,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-15 13:00:10</t>
+          <t>Timestamp: 2026-09-15 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19519</v>
+        <v>20019</v>
       </c>
     </row>
     <row r="3">
@@ -41190,11 +41190,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>21691</v>
+        <v>21991</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+1214</t>
+          <t>+1514</t>
         </is>
       </c>
     </row>
@@ -41535,11 +41535,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>32726</v>
+        <v>32776</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2146</t>
+          <t>+2196</t>
         </is>
       </c>
     </row>
@@ -41595,11 +41595,11 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>15794</v>
+        <v>15944</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+450</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-16 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -41757,7 +41757,7 @@
   <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -41778,11 +41778,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-16 13:00:10</t>
+          <t>Timestamp: 2026-09-16 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>11751</v>
+        <v>12001</v>
       </c>
     </row>
     <row r="3">
@@ -41910,7 +41910,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>SS Aiko Turbo Saetta</t>
+          <t>SS Aiko</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -41918,7 +41918,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -41974,11 +41974,11 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>13446</v>
+        <v>13496</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>+725</t>
+          <t>+775</t>
         </is>
       </c>
     </row>
@@ -42109,11 +42109,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>11258</v>
+        <v>11308</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+1856</t>
+          <t>+1906</t>
         </is>
       </c>
     </row>
@@ -42154,11 +42154,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>24327</v>
+        <v>24377</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+935</t>
+          <t>+985</t>
         </is>
       </c>
     </row>
@@ -42289,11 +42289,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>20113</v>
+        <v>20163</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1345</t>
+          <t>+1395</t>
         </is>
       </c>
     </row>
@@ -42364,11 +42364,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>34845</v>
+        <v>34895</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2069</t>
+          <t>+2119</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:00:12
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -61,6 +61,7 @@
     <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -42576,6 +42577,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-17 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>10208</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6735</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>16011</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+966</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>4065</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>38257</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1011</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1391</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6457</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>13796</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>24044</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+653</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>10600</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3414</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11012</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+746</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>3216</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>30683</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1421</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>12778</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+1470</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6586</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>26153</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1776</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>6642</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>18648</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+1763</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>8907</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>12123</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> cassanova98</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21361</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1198</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>630</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Brandal Lokajaya</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1472</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>16422</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>10335</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>36775</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+1880</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3120</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+232</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>17507</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+887</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>13990</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+348</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>9978</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+310</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>12033</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>1429</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1530</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+80</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>914</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+64</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>13747</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+632</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:10:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -42607,11 +42607,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-17 13:00:10</t>
+          <t>Timestamp: 2026-09-17 13:10:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10208</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
@@ -42938,11 +42938,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>12778</v>
+        <v>12828</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+1470</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>
@@ -42983,11 +42983,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>26153</v>
+        <v>26185</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+1776</t>
+          <t>+1808</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:30:31
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -42607,11 +42607,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-17 13:10:22</t>
+          <t>Timestamp: 2026-09-17 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>82</v>
+        <v>593</v>
       </c>
     </row>
     <row r="3">
@@ -42893,11 +42893,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>11012</v>
+        <v>11027</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+746</t>
+          <t>+761</t>
         </is>
       </c>
     </row>
@@ -43088,11 +43088,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>12123</v>
+        <v>12423</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -43118,11 +43118,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>21361</v>
+        <v>21552</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1198</t>
+          <t>+1389</t>
         </is>
       </c>
     </row>
@@ -43193,11 +43193,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>36775</v>
+        <v>36780</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+1880</t>
+          <t>+1885</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:40:39
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -42607,11 +42607,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-17 13:30:30</t>
+          <t>Timestamp: 2026-09-17 13:40:37</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>593</v>
+        <v>934</v>
       </c>
     </row>
     <row r="3">
@@ -42938,11 +42938,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>12828</v>
+        <v>12878</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+1520</t>
+          <t>+1570</t>
         </is>
       </c>
     </row>
@@ -42983,11 +42983,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>26185</v>
+        <v>26235</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+1808</t>
+          <t>+1858</t>
         </is>
       </c>
     </row>
@@ -43118,11 +43118,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>21552</v>
+        <v>21602</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1389</t>
+          <t>+1439</t>
         </is>
       </c>
     </row>
@@ -43193,11 +43193,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>36780</v>
+        <v>36821</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+1885</t>
+          <t>+1926</t>
         </is>
       </c>
     </row>
@@ -43253,11 +43253,11 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>17507</v>
+        <v>17657</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>+887</t>
+          <t>+1037</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-18 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -62,6 +62,7 @@
     <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="2026-09-18" sheetId="56" state="visible" r:id="rId56"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43405,6 +43406,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-18 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22916</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2598</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6735</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>16621</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>4345</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>39459</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1202</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1471</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+80</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2123</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6457</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>14583</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+787</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>25069</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>10600</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3905</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+491</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11589</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+562</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>3478</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+262</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>32539</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1856</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>14627</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+1749</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6586</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>28313</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+2078</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Carlos M$</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6642</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>19587</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+939</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8907</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>12730</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+307</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> cassanova98</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2129</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+356</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>23215</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1613</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1090</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Brandal Lokajaya</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>3026</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+1554</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>16422</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>10335</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>38739</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1918</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>3150</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+30</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>18239</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+582</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>14816</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+826</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>10178</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>13218</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+1185</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1529</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>964</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>14247</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-18 05:41:41
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -43436,11 +43436,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-18 13:30:23</t>
+          <t>Timestamp: 2026-09-18 13:41:40</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>80</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
@@ -43767,11 +43767,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>14632</v>
+        <v>14657</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+1754</t>
+          <t>+1779</t>
         </is>
       </c>
     </row>
@@ -43812,11 +43812,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>28313</v>
+        <v>28363</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+2078</t>
+          <t>+2128</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -63,6 +63,7 @@
     <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-09-18" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="2026-09-19" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44249,6 +44250,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-19 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2898</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6735</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>18222</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+1601</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>4345</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>41055</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1596</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1471</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2365</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+242</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6457</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>15884</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+1301</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>25897</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+828</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>10600</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3905</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>13443</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1854</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>3579</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+101</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>34364</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>14812</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+155</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6586</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>29053</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Carlos M$</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6642</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>21316</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1729</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>9185</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+278</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>12730</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> cassanova98</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2379</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>24602</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1387</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1090</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Brandal Lokajaya</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>4668</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+1617</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>16422</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>10458</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+123</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>40792</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>3400</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>19654</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+1415</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15116</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>10178</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>13518</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1730</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>14547</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 05:30:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -44280,7 +44280,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-19 13:00:10</t>
+          <t>Timestamp: 2026-09-19 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -44596,11 +44596,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>34364</v>
+        <v>34764</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+2200</t>
         </is>
       </c>
     </row>
@@ -44881,11 +44881,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>40792</v>
+        <v>40892</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+2028</t>
+          <t>+2128</t>
         </is>
       </c>
     </row>
@@ -44956,11 +44956,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>15116</v>
+        <v>15379</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+563</t>
         </is>
       </c>
     </row>
@@ -45016,11 +45016,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>13518</v>
+        <v>14099</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+881</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -64,6 +64,7 @@
     <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-09-18" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-09-19" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="2026-09-20" sheetId="58" state="visible" r:id="rId58"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45093,6 +45094,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-20 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>23193</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+20295</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>8925</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+2190</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>34681</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+16459</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>20028</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+15683</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>61197</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+20142</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>11323</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+9852</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>16322</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+16322</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>16914</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+14549</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>8658</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+2201</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>29140</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+13256</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>19337</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+19121</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>7967</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+7967</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>43352</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+17455</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>26321</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+15721</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>10501</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+6596</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>33203</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+19760</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>19413</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+15834</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>52881</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+18117</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>39139</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+24327</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>1270</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7706</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>54260</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+25207</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Carlos M$</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>15742</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+15722</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8642</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Nemo</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>39961</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+18645</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>13318</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+13318</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Hanagaki Takemichi</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>21663</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+20633</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>25474</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+16289</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>6381</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>14865</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+2135</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> cassanova98</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>21536</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+19157</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>44107</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+19505</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>11548</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+10458</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Brandal Lokajaya</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>25358</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+20690</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>32594</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+16172</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>29212</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+18754</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>44902</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+4010</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>11472</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+11472</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>18682</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+15282</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>6516</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+6516</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>37400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+17746</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>34816</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+19437</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>27328</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+17150</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>12244</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+11444</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Natsu Dragneel</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>4392</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Mydorya</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>6521</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>34844</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+20745</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>9932</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+8303</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>2190</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>18677</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+4130</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -45124,7 +45124,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-20 13:00:10</t>
+          <t>Timestamp: 2026-09-20 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -45856,7 +45856,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>SS Ruzzz.</t>
+          <t>Ryouza.</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -45864,7 +45864,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+17150</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>